<commit_message>
Update Service Deal AC repair website with latest changes
- Enhanced booking functionality with improved error handling
- Updated WhatsApp integration for post-booking communication
- Fixed server-side booking API with Excel data storage
- Updated contact information and branding
- Improved user experience with loading states and notifications
</commit_message>
<xml_diff>
--- a/bookings.xlsx
+++ b/bookings.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,9 +413,51 @@
         <v>Timestamp</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Test User</v>
+      </c>
+      <c r="B2" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="C2" t="str">
+        <v>AC Repair</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-03-09T10:04:22.007Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Test User</v>
+      </c>
+      <c r="B3" t="str">
+        <v>1234567890</v>
+      </c>
+      <c r="C3" t="str">
+        <v>AC Repair</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-03-09T10:09:42.541Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Atul</v>
+      </c>
+      <c r="B4" t="str">
+        <v>7706060100</v>
+      </c>
+      <c r="C4" t="str">
+        <v>repair</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-03-09T10:15:15.798Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>